<commit_message>
data: 0612 data update
</commit_message>
<xml_diff>
--- a/public/database/outsourcing.xlsx
+++ b/public/database/outsourcing.xlsx
@@ -1241,7 +1241,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1257,7 +1257,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="1">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1265,7 +1265,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1273,7 +1273,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="1">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1305,7 +1305,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -1329,7 +1329,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="1">
-        <v>33</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -1337,7 +1337,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="1">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:2">

</xml_diff>

<commit_message>
data: 0620 data update
</commit_message>
<xml_diff>
--- a/public/database/outsourcing.xlsx
+++ b/public/database/outsourcing.xlsx
@@ -1249,7 +1249,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="1">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1265,7 +1265,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1297,7 +1297,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1329,7 +1329,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="1">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -1337,7 +1337,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="1">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:2">

</xml_diff>